<commit_message>
små endringer i tegning
</commit_message>
<xml_diff>
--- a/TermProject/exponentiationfsm_state_table.xlsx
+++ b/TermProject/exponentiationfsm_state_table.xlsx
@@ -5,11 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="rsa_core_fsm" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Ark1" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="exponentsiation_fsm" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="45">
   <si>
     <t xml:space="preserve">Inputs</t>
   </si>
@@ -104,28 +104,58 @@
     <t xml:space="preserve">FINISHED</t>
   </si>
   <si>
+    <t xml:space="preserve">inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">States</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Action on signals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ready_out </t>
+  </si>
+  <si>
+    <t xml:space="preserve">load_result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valid_out </t>
+  </si>
+  <si>
     <t xml:space="preserve">current state</t>
   </si>
   <si>
     <t xml:space="preserve">next state</t>
   </si>
   <si>
-    <t xml:space="preserve">ready_out </t>
-  </si>
-  <si>
-    <t xml:space="preserve">load_result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valid_out </t>
-  </si>
-  <si>
     <t xml:space="preserve">reset</t>
   </si>
   <si>
     <t xml:space="preserve">counting</t>
   </si>
   <si>
+    <t xml:space="preserve">Counter = counter + 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">finished</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counter =  counter + 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if valid_out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r_reg &lt;= </t>
   </si>
 </sst>
 </file>
@@ -201,7 +231,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -216,6 +246,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -948,172 +982,310 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:G10"/>
+  <dimension ref="B2:K28"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="1" style="1" width="10.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.89"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="12.05"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.08"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="1" width="10.6"/>
+  </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E2" s="0" t="s">
+      <c r="B2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>28</v>
       </c>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="4"/>
+      <c r="K2" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>31</v>
+      <c r="C3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="0" t="n">
-        <v>0</v>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="0" t="n">
-        <v>0</v>
+      <c r="B5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="0" t="n">
-        <v>0</v>
+      <c r="B6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="0" t="n">
-        <v>0</v>
+      <c r="B7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="0" t="n">
-        <v>0</v>
+      <c r="B8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" s="0" t="n">
-        <v>1</v>
+      <c r="B9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" s="0" t="n">
-        <v>1</v>
+      <c r="B10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D27" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E28" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
oppdatert mer av tilstandstabell
</commit_message>
<xml_diff>
--- a/TermProject/exponentiationfsm_state_table.xlsx
+++ b/TermProject/exponentiationfsm_state_table.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="72">
   <si>
     <t xml:space="preserve">Inputs</t>
   </si>
@@ -215,10 +215,28 @@
     <t xml:space="preserve">S10[256]</t>
   </si>
   <si>
+    <t xml:space="preserve">S11</t>
+  </si>
+  <si>
     <t xml:space="preserve">S9[256]</t>
   </si>
   <si>
     <t xml:space="preserve">S8[256]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S6</t>
   </si>
 </sst>
 </file>
@@ -1142,8 +1160,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.13"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="30.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="12.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="9.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="20.38"/>
@@ -2294,6 +2312,9 @@
       <c r="B82" s="1" t="s">
         <v>63</v>
       </c>
+      <c r="D82" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E82" s="7" t="n">
         <v>0</v>
       </c>
@@ -2315,6 +2336,9 @@
         <v>1</v>
       </c>
       <c r="B83" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D83" s="8" t="s">
         <v>64</v>
       </c>
       <c r="E83" s="7" t="n">
@@ -2338,7 +2362,10 @@
         <v>0</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+      <c r="D84" s="8" t="s">
+        <v>64</v>
       </c>
       <c r="E84" s="7" t="n">
         <v>0</v>
@@ -2357,6 +2384,9 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D85" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E85" s="7" t="n">
         <v>0</v>
       </c>
@@ -2374,6 +2404,9 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D86" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E86" s="7" t="n">
         <v>0</v>
       </c>
@@ -2391,6 +2424,9 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D87" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E87" s="7" t="n">
         <v>0</v>
       </c>
@@ -2408,6 +2444,9 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D88" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E88" s="7" t="n">
         <v>0</v>
       </c>
@@ -2425,6 +2464,9 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D89" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E89" s="7" t="n">
         <v>0</v>
       </c>
@@ -2442,6 +2484,9 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D90" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="E90" s="7" t="n">
         <v>0</v>
       </c>
@@ -2459,6 +2504,9 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D91" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="E91" s="7" t="n">
         <v>0</v>
       </c>
@@ -2476,6 +2524,9 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D92" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="E92" s="7" t="n">
         <v>0</v>
       </c>
@@ -2493,6 +2544,9 @@
       </c>
     </row>
     <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D93" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="E93" s="7" t="n">
         <v>0</v>
       </c>
@@ -2510,6 +2564,9 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D94" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="E94" s="7" t="n">
         <v>0</v>
       </c>
@@ -2527,6 +2584,9 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D95" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="E95" s="7" t="n">
         <v>0</v>
       </c>
@@ -2544,6 +2604,9 @@
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D96" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="E96" s="7" t="n">
         <v>0</v>
       </c>
@@ -2561,6 +2624,9 @@
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D97" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="E97" s="7" t="n">
         <v>0</v>
       </c>
@@ -2578,6 +2644,9 @@
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D98" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E98" s="1" t="n">
         <v>1</v>
       </c>
@@ -2595,6 +2664,9 @@
       </c>
     </row>
     <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D99" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E99" s="1" t="n">
         <v>1</v>
       </c>
@@ -2612,6 +2684,9 @@
       </c>
     </row>
     <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D100" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E100" s="1" t="n">
         <v>1</v>
       </c>
@@ -2629,6 +2704,9 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D101" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E101" s="1" t="n">
         <v>1</v>
       </c>
@@ -2646,6 +2724,9 @@
       </c>
     </row>
     <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D102" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="E102" s="1" t="n">
         <v>1</v>
       </c>
@@ -2663,6 +2744,9 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D103" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E103" s="1" t="n">
         <v>1</v>
       </c>
@@ -2680,6 +2764,9 @@
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D104" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="E104" s="1" t="n">
         <v>1</v>
       </c>
@@ -2697,6 +2784,9 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D105" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E105" s="1" t="n">
         <v>1</v>
       </c>
@@ -2714,6 +2804,9 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D106" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E106" s="1" t="n">
         <v>1</v>
       </c>
@@ -2731,6 +2824,9 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D107" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E107" s="1" t="n">
         <v>1</v>
       </c>
@@ -2748,6 +2844,9 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D108" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E108" s="1" t="n">
         <v>1</v>
       </c>
@@ -2765,6 +2864,9 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D109" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E109" s="1" t="n">
         <v>1</v>
       </c>
@@ -2782,6 +2884,9 @@
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D110" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="E110" s="1" t="n">
         <v>1</v>
       </c>
@@ -2799,6 +2904,9 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D111" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E111" s="1" t="n">
         <v>1</v>
       </c>
@@ -2816,6 +2924,9 @@
       </c>
     </row>
     <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D112" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="E112" s="1" t="n">
         <v>1</v>
       </c>
@@ -2833,6 +2944,9 @@
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D113" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E113" s="1" t="n">
         <v>1</v>
       </c>

</xml_diff>